<commit_message>
chore(workbook): commit the filled workbook the 2026-10-12 import regenerated
fill_ternarios.py rewrote it at 13:19, after 1089467, inside bin/import-lle; the
committed copy predated d074140's leaner-vial rule. 32 cached aqueous cells
(AD-AG) in blocks A, B, D, H change; no input cell does.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sistemas ternarios_MF_filled.xlsx
+++ b/Sistemas ternarios_MF_filled.xlsx
@@ -1520,16 +1520,16 @@
         <v>2</v>
       </c>
       <c r="AD7" s="31" t="n">
-        <v>0.00133391210031924</v>
+        <v>0.00131439593254686</v>
       </c>
       <c r="AE7" s="31" t="n">
-        <v>0.000685912957483989</v>
+        <v>0.000331876406245623</v>
       </c>
       <c r="AF7" s="31" t="n">
-        <v>0.000801557358974884</v>
+        <v>0.000429268908006592</v>
       </c>
       <c r="AG7" s="31" t="n">
-        <v>0.997178617583222</v>
+        <v>0.997924458753201</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1729,16 +1729,16 @@
         <v>3</v>
       </c>
       <c r="AD9" s="31" t="n">
-        <v>0.0240256555085348</v>
+        <v>0.0242128859067119</v>
       </c>
       <c r="AE9" s="31" t="n">
-        <v>2.58847976788953E-005</v>
+        <v>2.1224264005602E-005</v>
       </c>
       <c r="AF9" s="31" t="n">
-        <v>4.96116341927225E-005</v>
+        <v>4.38811348964189E-005</v>
       </c>
       <c r="AG9" s="31" t="n">
-        <v>0.975898848059594</v>
+        <v>0.975722008694386</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2729,16 +2729,16 @@
       </c>
       <c r="AB19" s="2"/>
       <c r="AD19" s="0" t="n">
-        <v>0.0083912019804683</v>
+        <v>0.00786374369982345</v>
       </c>
       <c r="AE19" s="0" t="n">
-        <v>0.000773677351107489</v>
+        <v>0.000335604906130558</v>
       </c>
       <c r="AF19" s="0" t="n">
-        <v>0.000945970661007499</v>
+        <v>0.000486851403368356</v>
       </c>
       <c r="AG19" s="0" t="n">
-        <v>0.989889150007417</v>
+        <v>0.991313799990678</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3772,16 +3772,16 @@
         <v>0.962892579742591</v>
       </c>
       <c r="AD5" s="0" t="n">
-        <v>0.0269449351828853</v>
+        <v>0.0249102993464579</v>
       </c>
       <c r="AE5" s="0" t="n">
-        <v>6.11845024389588E-005</v>
+        <v>2.33107578428212E-005</v>
       </c>
       <c r="AF5" s="0" t="n">
-        <v>7.11999726022893E-005</v>
+        <v>3.11945685660548E-005</v>
       </c>
       <c r="AG5" s="0" t="n">
-        <v>0.972922680342074</v>
+        <v>0.975035195327133</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5073,16 +5073,16 @@
         <v>0.998103391430224</v>
       </c>
       <c r="AD19" s="0" t="n">
-        <v>0.00903120686880268</v>
+        <v>0.008776458612092</v>
       </c>
       <c r="AE19" s="0" t="n">
-        <v>0.000879942293655311</v>
+        <v>0.000389405566648141</v>
       </c>
       <c r="AF19" s="0" t="n">
-        <v>0.000803088908771208</v>
+        <v>0.000286059240735268</v>
       </c>
       <c r="AG19" s="0" t="n">
-        <v>0.989285761928771</v>
+        <v>0.990548076580525</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5445,16 +5445,16 @@
         <v>0.998622949499804</v>
       </c>
       <c r="AD23" s="0" t="n">
-        <v>0.0209087059304334</v>
+        <v>0.0203487415232242</v>
       </c>
       <c r="AE23" s="0" t="n">
-        <v>0.000302432844891912</v>
+        <v>0.000205702317551325</v>
       </c>
       <c r="AF23" s="0" t="n">
-        <v>0.000316434224783248</v>
+        <v>0.000216708489771156</v>
       </c>
       <c r="AG23" s="0" t="n">
-        <v>0.978472426999892</v>
+        <v>0.979228847669453</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9791,16 +9791,16 @@
         <v>1.00823753359508</v>
       </c>
       <c r="AD21" s="0" t="n">
-        <v>0.00808221542284589</v>
+        <v>0.00726214373206045</v>
       </c>
       <c r="AE21" s="0" t="n">
-        <v>0.00393072909126719</v>
+        <v>0.00289929210117323</v>
       </c>
       <c r="AF21" s="0" t="n">
-        <v>0.0045128072826791</v>
+        <v>0.00343251162688846</v>
       </c>
       <c r="AG21" s="0" t="n">
-        <v>0.983474248203208</v>
+        <v>0.986406052539878</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15635,16 +15635,16 @@
         <v>0.993981804136749</v>
       </c>
       <c r="AD9" s="0" t="n">
-        <v>0.025030281549823</v>
+        <v>0.0252102595450379</v>
       </c>
       <c r="AE9" s="0" t="n">
-        <v>0.00012056508831252</v>
+        <v>8.04924118460484E-005</v>
       </c>
       <c r="AF9" s="0" t="n">
-        <v>5.94563422035077E-005</v>
+        <v>1.94615075386359E-005</v>
       </c>
       <c r="AG9" s="0" t="n">
-        <v>0.974789697019661</v>
+        <v>0.974689786535578</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>